<commit_message>
Add admin dashboard and React UI
</commit_message>
<xml_diff>
--- a/API/bin/Debug/net8.0/mydiet.xlsx
+++ b/API/bin/Debug/net8.0/mydiet.xlsx
@@ -43,6 +43,12 @@
   </x:si>
   <x:si>
     <x:t>John</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-13T21:02:12.7280000Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Test</x:t>
   </x:si>
   <x:si>
     <x:t>WeightKg</x:t>
@@ -453,6 +459,108 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:5">
+      <x:c r="A7" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D7" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:5">
+      <x:c r="A8" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:5">
+      <x:c r="A9" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D9" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -478,7 +586,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>4</x:v>
@@ -506,7 +614,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>